<commit_message>
tree view in docs
</commit_message>
<xml_diff>
--- a/AhMen Doc Templates/AhMen Client Data and Docs Template.xlsx
+++ b/AhMen Doc Templates/AhMen Client Data and Docs Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/motticohen/Desktop/invoice_master_dashboard/AhMen Doc Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E882BB7A-B302-764F-9639-2BDC486FFC2C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BB58532-66BE-C747-A255-31D2F0A40543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="500" windowWidth="27160" windowHeight="28300" activeTab="5" xr2:uid="{B5763DD8-C14C-9E43-BCE3-8FC2FCC62202}"/>
+    <workbookView xWindow="60" yWindow="500" windowWidth="27160" windowHeight="28300" activeTab="2" xr2:uid="{B5763DD8-C14C-9E43-BCE3-8FC2FCC62202}"/>
   </bookViews>
   <sheets>
     <sheet name="Client Data" sheetId="3" r:id="rId1"/>
@@ -3190,7 +3190,7 @@
     <xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="32" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="14" fontId="22" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -5465,17 +5465,17 @@
       <c r="E72" s="107"/>
       <c r="F72" s="107"/>
     </row>
-    <row r="73" spans="2:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="73" spans="2:6" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B73" s="64" t="s">
         <v>147</v>
       </c>
-      <c r="D73" s="107" t="s">
+      <c r="D73" s="52" t="s">
         <v>196</v>
       </c>
       <c r="E73" s="107"/>
       <c r="F73" s="107"/>
     </row>
-    <row r="74" spans="2:6" ht="20" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="74" spans="2:6" ht="20" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B74" s="64" t="s">
         <v>146</v>
       </c>

</xml_diff>

<commit_message>
file management tab is back
</commit_message>
<xml_diff>
--- a/AhMen Doc Templates/AhMen Client Data and Docs Template.xlsx
+++ b/AhMen Doc Templates/AhMen Client Data and Docs Template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/motticohen/Desktop/invoice_master_dashboard/AhMen Doc Templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1BB58532-66BE-C747-A255-31D2F0A40543}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B4411C0-AD9C-ED4A-8DC1-7D9B536F1C52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="60" yWindow="500" windowWidth="27160" windowHeight="28300" activeTab="2" xr2:uid="{B5763DD8-C14C-9E43-BCE3-8FC2FCC62202}"/>
+    <workbookView xWindow="60" yWindow="500" windowWidth="27160" windowHeight="28300" activeTab="1" xr2:uid="{B5763DD8-C14C-9E43-BCE3-8FC2FCC62202}"/>
   </bookViews>
   <sheets>
     <sheet name="Client Data" sheetId="3" r:id="rId1"/>
@@ -28,7 +28,7 @@
     <definedName name="_xlnm.Print_Area" localSheetId="1">Quote!$A$1:$J$43</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="3">'T&amp;Cs'!$A$1:$H$72</definedName>
   </definedNames>
-  <calcPr calcId="191029" fullCalcOnLoad="1" calcOnSave="1"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -3165,6 +3165,9 @@
     <xf numFmtId="167" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="14" fontId="22" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -3189,9 +3192,6 @@
     </xf>
     <xf numFmtId="0" fontId="52" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="14" fontId="22" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -4209,17 +4209,17 @@
       <c r="B1" s="2"/>
     </row>
     <row r="2" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B2" s="118" t="s">
+      <c r="B2" s="119" t="s">
         <v>30</v>
       </c>
-      <c r="C2" s="118"/>
+      <c r="C2" s="119"/>
       <c r="D2" s="85"/>
       <c r="E2" s="86"/>
       <c r="F2" s="85"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B3" s="118"/>
-      <c r="C3" s="118"/>
+      <c r="B3" s="119"/>
+      <c r="C3" s="119"/>
       <c r="D3" s="85"/>
       <c r="E3" s="86"/>
       <c r="F3" s="85"/>
@@ -4228,10 +4228,10 @@
       <c r="B4" s="7"/>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B5" s="119" t="s">
+      <c r="B5" s="120" t="s">
         <v>32</v>
       </c>
-      <c r="C5" s="119"/>
+      <c r="C5" s="120"/>
       <c r="D5" s="26"/>
       <c r="E5" s="30" t="s">
         <v>31</v>
@@ -4246,7 +4246,7 @@
       <c r="D6" s="26"/>
       <c r="E6" s="27">
         <f ca="1">TODAY()</f>
-        <v>45925</v>
+        <v>45926</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -4371,12 +4371,12 @@
       <c r="H21" s="3"/>
     </row>
     <row r="22" spans="2:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="120" t="s">
+      <c r="B22" s="121" t="s">
         <v>152</v>
       </c>
-      <c r="C22" s="120"/>
-      <c r="D22" s="120"/>
-      <c r="E22" s="120"/>
+      <c r="C22" s="121"/>
+      <c r="D22" s="121"/>
+      <c r="E22" s="121"/>
       <c r="F22" s="117" t="str">
         <f>'Client Data'!B28</f>
         <v>EXTRA_FEES</v>
@@ -4407,12 +4407,12 @@
       <c r="I24" s="9"/>
     </row>
     <row r="25" spans="2:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B25" s="120" t="s">
+      <c r="B25" s="121" t="s">
         <v>162</v>
       </c>
-      <c r="C25" s="120"/>
-      <c r="D25" s="120"/>
-      <c r="E25" s="120"/>
+      <c r="C25" s="121"/>
+      <c r="D25" s="121"/>
+      <c r="E25" s="121"/>
       <c r="F25" s="3"/>
       <c r="G25" s="3"/>
       <c r="H25" s="3"/>
@@ -4611,20 +4611,20 @@
       <c r="E1" s="2"/>
     </row>
     <row r="2" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="118" t="s">
+      <c r="B2" s="119" t="s">
         <v>34</v>
       </c>
-      <c r="C2" s="118"/>
-      <c r="D2" s="118"/>
-      <c r="E2" s="118"/>
-      <c r="F2" s="118"/>
+      <c r="C2" s="119"/>
+      <c r="D2" s="119"/>
+      <c r="E2" s="119"/>
+      <c r="F2" s="119"/>
     </row>
     <row r="3" spans="1:9" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="118"/>
-      <c r="C3" s="118"/>
-      <c r="D3" s="118"/>
-      <c r="E3" s="118"/>
-      <c r="F3" s="118"/>
+      <c r="B3" s="119"/>
+      <c r="C3" s="119"/>
+      <c r="D3" s="119"/>
+      <c r="E3" s="119"/>
+      <c r="F3" s="119"/>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B4" s="7"/>
@@ -4633,11 +4633,11 @@
       <c r="E4" s="7"/>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B5" s="123"/>
-      <c r="C5" s="123"/>
-      <c r="D5" s="123"/>
-      <c r="E5" s="123"/>
-      <c r="F5" s="123"/>
+      <c r="B5" s="124"/>
+      <c r="C5" s="124"/>
+      <c r="D5" s="124"/>
+      <c r="E5" s="124"/>
+      <c r="F5" s="124"/>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.2">
       <c r="B6" s="42"/>
@@ -4704,19 +4704,19 @@
       <c r="F12" s="43"/>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="B13" s="124"/>
-      <c r="C13" s="124"/>
-      <c r="D13" s="124"/>
-      <c r="E13" s="124"/>
-      <c r="F13" s="124"/>
+      <c r="B13" s="125"/>
+      <c r="C13" s="125"/>
+      <c r="D13" s="125"/>
+      <c r="E13" s="125"/>
+      <c r="F13" s="125"/>
     </row>
     <row r="14" spans="1:9" ht="20" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="48"/>
-      <c r="B14" s="121" t="s">
+      <c r="B14" s="122" t="s">
         <v>36</v>
       </c>
-      <c r="C14" s="121"/>
-      <c r="D14" s="121"/>
+      <c r="C14" s="122"/>
+      <c r="D14" s="122"/>
       <c r="E14" s="88"/>
       <c r="F14" s="89"/>
       <c r="G14" s="90"/>
@@ -4786,11 +4786,11 @@
         <v>127</v>
       </c>
       <c r="C19" s="49"/>
-      <c r="D19" s="125" t="str">
+      <c r="D19" s="126" t="str">
         <f>'Client Data'!B14</f>
         <v>EVENT_DATE</v>
       </c>
-      <c r="E19" s="125"/>
+      <c r="E19" s="126"/>
       <c r="F19" s="56"/>
       <c r="G19" s="56"/>
       <c r="H19" s="56"/>
@@ -4947,11 +4947,11 @@
     </row>
     <row r="30" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="48"/>
-      <c r="B30" s="121" t="s">
+      <c r="B30" s="122" t="s">
         <v>39</v>
       </c>
-      <c r="C30" s="121"/>
-      <c r="D30" s="121"/>
+      <c r="C30" s="122"/>
+      <c r="D30" s="122"/>
       <c r="E30" s="88"/>
       <c r="F30" s="89"/>
       <c r="G30" s="90"/>
@@ -5072,11 +5072,11 @@
     </row>
     <row r="39" spans="1:21" ht="20" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="48"/>
-      <c r="B39" s="122" t="s">
+      <c r="B39" s="123" t="s">
         <v>40</v>
       </c>
-      <c r="C39" s="122"/>
-      <c r="D39" s="122"/>
+      <c r="C39" s="123"/>
+      <c r="D39" s="123"/>
       <c r="E39" s="88"/>
       <c r="F39" s="89"/>
       <c r="G39" s="90"/>
@@ -5479,9 +5479,9 @@
       <c r="B74" s="64" t="s">
         <v>146</v>
       </c>
-      <c r="D74" s="127">
+      <c r="D74" s="118">
         <f ca="1">TODAY()</f>
-        <v>45925</v>
+        <v>45926</v>
       </c>
       <c r="E74" s="71"/>
     </row>
@@ -5768,19 +5768,19 @@
       <c r="E1" s="2"/>
     </row>
     <row r="2" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="126" t="s">
+      <c r="B2" s="127" t="s">
         <v>161</v>
       </c>
-      <c r="C2" s="126"/>
-      <c r="D2" s="126"/>
-      <c r="E2" s="126"/>
+      <c r="C2" s="127"/>
+      <c r="D2" s="127"/>
+      <c r="E2" s="127"/>
       <c r="F2" s="85"/>
     </row>
     <row r="3" spans="2:7" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="126"/>
-      <c r="C3" s="126"/>
-      <c r="D3" s="126"/>
-      <c r="E3" s="126"/>
+      <c r="B3" s="127"/>
+      <c r="C3" s="127"/>
+      <c r="D3" s="127"/>
+      <c r="E3" s="127"/>
       <c r="F3" s="85"/>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.2">
@@ -6508,17 +6508,17 @@
       <c r="B1" s="2"/>
     </row>
     <row r="2" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B2" s="118" t="s">
+      <c r="B2" s="119" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="118"/>
+      <c r="C2" s="119"/>
       <c r="D2" s="85"/>
       <c r="E2" s="86"/>
       <c r="F2" s="85"/>
     </row>
     <row r="3" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B3" s="118"/>
-      <c r="C3" s="118"/>
+      <c r="B3" s="119"/>
+      <c r="C3" s="119"/>
       <c r="D3" s="85"/>
       <c r="E3" s="86"/>
       <c r="F3" s="85"/>
@@ -6527,10 +6527,10 @@
       <c r="B4" s="7"/>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B5" s="119" t="s">
+      <c r="B5" s="120" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="119"/>
+      <c r="C5" s="120"/>
       <c r="D5" s="26"/>
       <c r="E5" s="30" t="s">
         <v>23</v>
@@ -6545,7 +6545,7 @@
       <c r="D6" s="26"/>
       <c r="E6" s="27">
         <f ca="1">TODAY()</f>
-        <v>45925</v>
+        <v>45926</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -6674,12 +6674,12 @@
       <c r="H21" s="3"/>
     </row>
     <row r="22" spans="2:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="120" t="s">
+      <c r="B22" s="121" t="s">
         <v>152</v>
       </c>
-      <c r="C22" s="120"/>
-      <c r="D22" s="120"/>
-      <c r="E22" s="120"/>
+      <c r="C22" s="121"/>
+      <c r="D22" s="121"/>
+      <c r="E22" s="121"/>
       <c r="F22" s="117" t="str">
         <f>'Client Data'!B28</f>
         <v>EXTRA_FEES</v>
@@ -6711,12 +6711,12 @@
     </row>
     <row r="25" spans="2:9" ht="20" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="26" spans="2:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B26" s="120" t="s">
+      <c r="B26" s="121" t="s">
         <v>160</v>
       </c>
-      <c r="C26" s="120"/>
-      <c r="D26" s="120"/>
-      <c r="E26" s="120"/>
+      <c r="C26" s="121"/>
+      <c r="D26" s="121"/>
+      <c r="E26" s="121"/>
       <c r="F26" s="3"/>
       <c r="G26" s="3"/>
       <c r="H26" s="3"/>
@@ -6794,7 +6794,7 @@
       </c>
       <c r="C33" s="15">
         <f ca="1">TODAY()</f>
-        <v>45925</v>
+        <v>45926</v>
       </c>
       <c r="I33" s="6"/>
     </row>
@@ -6911,17 +6911,17 @@
       <c r="B1" s="2"/>
     </row>
     <row r="2" spans="2:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B2" s="118" t="s">
+      <c r="B2" s="119" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="118"/>
+      <c r="C2" s="119"/>
       <c r="D2" s="85"/>
       <c r="E2" s="86"/>
       <c r="F2" s="85"/>
     </row>
     <row r="3" spans="2:8" ht="16" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B3" s="118"/>
-      <c r="C3" s="118"/>
+      <c r="B3" s="119"/>
+      <c r="C3" s="119"/>
       <c r="D3" s="85"/>
       <c r="E3" s="86"/>
       <c r="F3" s="85"/>
@@ -6930,10 +6930,10 @@
       <c r="B4" s="7"/>
     </row>
     <row r="5" spans="2:8" x14ac:dyDescent="0.2">
-      <c r="B5" s="119" t="s">
+      <c r="B5" s="120" t="s">
         <v>22</v>
       </c>
-      <c r="C5" s="119"/>
+      <c r="C5" s="120"/>
       <c r="E5" s="30" t="s">
         <v>23</v>
       </c>
@@ -7073,12 +7073,12 @@
       <c r="I21" s="105"/>
     </row>
     <row r="22" spans="2:9" ht="20" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B22" s="120" t="s">
+      <c r="B22" s="121" t="s">
         <v>152</v>
       </c>
-      <c r="C22" s="120"/>
-      <c r="D22" s="120"/>
-      <c r="E22" s="120"/>
+      <c r="C22" s="121"/>
+      <c r="D22" s="121"/>
+      <c r="E22" s="121"/>
       <c r="F22" s="117" t="str">
         <f>'Client Data'!B28</f>
         <v>EXTRA_FEES</v>

</xml_diff>